<commit_message>
chore: update address book from website
</commit_message>
<xml_diff>
--- a/data/address-book.xlsx
+++ b/data/address-book.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kevin\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{43CA2712-3B86-4253-8C08-E2017C2D4591}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{003D299A-01BA-4D0B-A225-903052512865}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4320" yWindow="2775" windowWidth="21600" windowHeight="11295" xr2:uid="{719AF457-8665-40AE-9ECA-E2C783C5C2E0}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="68">
   <si>
     <t>ManhACE</t>
   </si>
@@ -102,6 +102,147 @@
   </si>
   <si>
     <t>0x8Dcaeb54Ebc684F924B2ae285281c98569E02326</t>
+  </si>
+  <si>
+    <t>EatShoes</t>
+  </si>
+  <si>
+    <t>0x43E019261b6C627fDdF91c8012AcC9F0C56e99c7</t>
+  </si>
+  <si>
+    <t>kakakakakak1</t>
+  </si>
+  <si>
+    <t>IUnar</t>
+  </si>
+  <si>
+    <t>0xE9E5e18DcB7932188f863d421c7aB8491a021175</t>
+  </si>
+  <si>
+    <t>Pokerman</t>
+  </si>
+  <si>
+    <t>0x7109670b65c1aeECb251D67407Af8cDF1e001185</t>
+  </si>
+  <si>
+    <t>DevilCase</t>
+  </si>
+  <si>
+    <t>o8888888</t>
+  </si>
+  <si>
+    <t>0x940Fbb99e06A4eDBd403ec2BdaC652F6e5eadda3</t>
+  </si>
+  <si>
+    <t>muuame</t>
+  </si>
+  <si>
+    <t>0x76daf610E09B31407244841e2A97682a32f32463</t>
+  </si>
+  <si>
+    <t>Lightbringer</t>
+  </si>
+  <si>
+    <t>0x99561e3080385C907c4A9B4bbB944508E8d1D15e</t>
+  </si>
+  <si>
+    <t>Osora</t>
+  </si>
+  <si>
+    <t>0x01e11d2925519f6C84EA49B6809f3D34b87a43Df</t>
+  </si>
+  <si>
+    <t>asdwqa12</t>
+  </si>
+  <si>
+    <t>0xA533F7729940DD9402da699aa8a9bD3281181FfC</t>
+  </si>
+  <si>
+    <t>Number17</t>
+  </si>
+  <si>
+    <t>0xbD015CC6F657D0D2c54dE363A9117a7f2db147A1</t>
+  </si>
+  <si>
+    <t>magisa</t>
+  </si>
+  <si>
+    <t>0x6f6E91a883A9Ec32068302a4051B27C57E376A48</t>
+  </si>
+  <si>
+    <t>MrKun</t>
+  </si>
+  <si>
+    <t>0xcb5C82d2fd95C35d4CAe44a2a5CD44C9b1201A87</t>
+  </si>
+  <si>
+    <t>INurseI</t>
+  </si>
+  <si>
+    <t>0xbF543fB6fe42f1c54A01385298c29D3Fba735951</t>
+  </si>
+  <si>
+    <t>Mitsuya</t>
+  </si>
+  <si>
+    <t>0xA5a0FeABD47B1865ba0a402abcfC810a7A560d06</t>
+  </si>
+  <si>
+    <t>ShadowSAMA</t>
+  </si>
+  <si>
+    <t>0x1db18A653bd7C6C2dc899933340B7a960b451399</t>
+  </si>
+  <si>
+    <t>ouwen110</t>
+  </si>
+  <si>
+    <t>0x37CA68Bcd9fd3f13CB732a3307ed64233F96a02d</t>
+  </si>
+  <si>
+    <t>NFT188</t>
+  </si>
+  <si>
+    <t>0x34219BDBfDcB233FCe08185724435fDd40E89929</t>
+  </si>
+  <si>
+    <t>KCOF</t>
+  </si>
+  <si>
+    <t>0x8E804BD15403d74C294752D66d970744876C5146</t>
+  </si>
+  <si>
+    <t>SoLUK</t>
+  </si>
+  <si>
+    <t>0x9bCeE51c0AEd896CAAb5fb6B7FB6630D1101Edd8</t>
+  </si>
+  <si>
+    <t>xQvQx</t>
+  </si>
+  <si>
+    <t>0xdf01a3312df58fA7B689Ce3fa1eFd9c0422171Bf</t>
+  </si>
+  <si>
+    <t>dXwXb</t>
+  </si>
+  <si>
+    <t>0xD8cc71d298F3A6f3D497357963Ac4723fc81FB8e</t>
+  </si>
+  <si>
+    <t>kappy</t>
+  </si>
+  <si>
+    <t>0xD63E33fB919d4dC190aD5c980DF71d3aF334DcA1</t>
+  </si>
+  <si>
+    <t>JBJOuO</t>
+  </si>
+  <si>
+    <t>0xB1cc3f69F8A6C965893B0398ab857475F367d2f1</t>
+  </si>
+  <si>
+    <t>chan9q</t>
   </si>
 </sst>
 </file>
@@ -485,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21573F96-787D-43CE-A4C4-3589456289B8}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B36"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -576,6 +717,206 @@
         <v>20</v>
       </c>
     </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>26</v>
+      </c>
+      <c r="B15" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>28</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>29</v>
+      </c>
+      <c r="B17" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>31</v>
+      </c>
+      <c r="B18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>37</v>
+      </c>
+      <c r="B21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>39</v>
+      </c>
+      <c r="B22" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>41</v>
+      </c>
+      <c r="B23" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>43</v>
+      </c>
+      <c r="B24" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>45</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B26" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>49</v>
+      </c>
+      <c r="B27" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>51</v>
+      </c>
+      <c r="B28" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>53</v>
+      </c>
+      <c r="B29" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>55</v>
+      </c>
+      <c r="B30" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>59</v>
+      </c>
+      <c r="B32" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>63</v>
+      </c>
+      <c r="B34" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>65</v>
+      </c>
+      <c r="B35" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>67</v>
+      </c>
+      <c r="B36" t="s">
+        <v>46</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>